<commit_message>
Kc de literatura (FAO-56) para cacau e tabaco (v6.1)
- TABACO: curva FAO-56 (Tabela 12) - Kc_ini 0,35 / Kc_mid 1,15 / Kc_end 0,90,
  fases 20/30/30/30
- CACAU: Kc de literatura ~1,00 constante (perene, dossel/sombra); editavel
  em CURVAS_KC. Sai de PENDENTE.

Validado: 9.303 celulas, zero erros. Recalculo ao abrir.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ytrvvbkWKcC1Fp4Ydm9J6
</commit_message>
<xml_diff>
--- a/Manejo_Irrigacao_Karitel_RDM.xlsx
+++ b/Manejo_Irrigacao_Karitel_RDM.xlsx
@@ -748,7 +748,7 @@
     <row r="11" ht="34" customHeight="1">
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>PENDENCIAS:  Cacau sem curva de Kc; variedade fora da lista usa classe padrao (edite a coluna Classe).</t>
+          <t>LITERATURA:  Tabaco e cacau usam Kc de LITERATURA (FAO-56): tabaco 0,35/1,15/0,90; cacau ~1,00 constante (perene). Edite em CURVAS_KC.</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
         <v/>
       </c>
       <c r="I6" s="12">
-        <f>IF($T6="","PENDENTE",IF($G6="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H6,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T6,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T6="","PENDENTE",IF($G6="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H6,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T6,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J6" s="13">
@@ -1211,7 +1211,7 @@
         <v/>
       </c>
       <c r="I7" s="12">
-        <f>IF($T7="","PENDENTE",IF($G7="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H7,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T7,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T7="","PENDENTE",IF($G7="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H7,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T7,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J7" s="13">
@@ -1298,7 +1298,7 @@
         <v/>
       </c>
       <c r="I8" s="12">
-        <f>IF($T8="","PENDENTE",IF($G8="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H8,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T8,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T8="","PENDENTE",IF($G8="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H8,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T8,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J8" s="13">
@@ -1385,7 +1385,7 @@
         <v/>
       </c>
       <c r="I9" s="12">
-        <f>IF($T9="","PENDENTE",IF($G9="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H9,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T9,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T9="","PENDENTE",IF($G9="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H9,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T9,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J9" s="13">
@@ -1472,7 +1472,7 @@
         <v/>
       </c>
       <c r="I10" s="12">
-        <f>IF($T10="","PENDENTE",IF($G10="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H10,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T10,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T10="","PENDENTE",IF($G10="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H10,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T10,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J10" s="13">
@@ -1559,7 +1559,7 @@
         <v/>
       </c>
       <c r="I11" s="12">
-        <f>IF($T11="","PENDENTE",IF($G11="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H11,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T11,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T11="","PENDENTE",IF($G11="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H11,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T11,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J11" s="13">
@@ -1646,7 +1646,7 @@
         <v/>
       </c>
       <c r="I12" s="12">
-        <f>IF($T12="","PENDENTE",IF($G12="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H12,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T12,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T12="","PENDENTE",IF($G12="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H12,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T12,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J12" s="13">
@@ -1733,7 +1733,7 @@
         <v/>
       </c>
       <c r="I13" s="12">
-        <f>IF($T13="","PENDENTE",IF($G13="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H13,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T13,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T13="","PENDENTE",IF($G13="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H13,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T13,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J13" s="13">
@@ -1820,7 +1820,7 @@
         <v/>
       </c>
       <c r="I14" s="12">
-        <f>IF($T14="","PENDENTE",IF($G14="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H14,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T14,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T14="","PENDENTE",IF($G14="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H14,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T14,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J14" s="13">
@@ -1907,7 +1907,7 @@
         <v/>
       </c>
       <c r="I15" s="12">
-        <f>IF($T15="","PENDENTE",IF($G15="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H15,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T15,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T15="","PENDENTE",IF($G15="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H15,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T15,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J15" s="13">
@@ -1994,7 +1994,7 @@
         <v/>
       </c>
       <c r="I16" s="12">
-        <f>IF($T16="","PENDENTE",IF($G16="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H16,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T16,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T16="","PENDENTE",IF($G16="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H16,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T16,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J16" s="13">
@@ -2081,7 +2081,7 @@
         <v/>
       </c>
       <c r="I17" s="12">
-        <f>IF($T17="","PENDENTE",IF($G17="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H17,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T17,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T17="","PENDENTE",IF($G17="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H17,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T17,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J17" s="13">
@@ -2168,7 +2168,7 @@
         <v/>
       </c>
       <c r="I18" s="12">
-        <f>IF($T18="","PENDENTE",IF($G18="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H18,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T18,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T18="","PENDENTE",IF($G18="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H18,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T18,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J18" s="13">
@@ -2255,7 +2255,7 @@
         <v/>
       </c>
       <c r="I19" s="12">
-        <f>IF($T19="","PENDENTE",IF($G19="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H19,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T19,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T19="","PENDENTE",IF($G19="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H19,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T19,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J19" s="13">
@@ -2342,7 +2342,7 @@
         <v/>
       </c>
       <c r="I20" s="12">
-        <f>IF($T20="","PENDENTE",IF($G20="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H20,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T20,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T20="","PENDENTE",IF($G20="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H20,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T20,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J20" s="13">
@@ -2429,7 +2429,7 @@
         <v/>
       </c>
       <c r="I21" s="12">
-        <f>IF($T21="","PENDENTE",IF($G21="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H21,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T21,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T21="","PENDENTE",IF($G21="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H21,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T21,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J21" s="13">
@@ -2516,7 +2516,7 @@
         <v/>
       </c>
       <c r="I22" s="12">
-        <f>IF($T22="","PENDENTE",IF($G22="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H22,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T22,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T22="","PENDENTE",IF($G22="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H22,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T22,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J22" s="13">
@@ -2603,7 +2603,7 @@
         <v/>
       </c>
       <c r="I23" s="12">
-        <f>IF($T23="","PENDENTE",IF($G23="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H23,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T23,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T23="","PENDENTE",IF($G23="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H23,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T23,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J23" s="13">
@@ -2690,7 +2690,7 @@
         <v/>
       </c>
       <c r="I24" s="12">
-        <f>IF($T24="","PENDENTE",IF($G24="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H24,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T24,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T24="","PENDENTE",IF($G24="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H24,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T24,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J24" s="13">
@@ -2777,7 +2777,7 @@
         <v/>
       </c>
       <c r="I25" s="12">
-        <f>IF($T25="","PENDENTE",IF($G25="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H25,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T25,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T25="","PENDENTE",IF($G25="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H25,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T25,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J25" s="13">
@@ -2864,7 +2864,7 @@
         <v/>
       </c>
       <c r="I26" s="12">
-        <f>IF($T26="","PENDENTE",IF($G26="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H26,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T26,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T26="","PENDENTE",IF($G26="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H26,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T26,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J26" s="13">
@@ -2951,7 +2951,7 @@
         <v/>
       </c>
       <c r="I27" s="12">
-        <f>IF($T27="","PENDENTE",IF($G27="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H27,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T27,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T27="","PENDENTE",IF($G27="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H27,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T27,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J27" s="13">
@@ -3038,7 +3038,7 @@
         <v/>
       </c>
       <c r="I28" s="12">
-        <f>IF($T28="","PENDENTE",IF($G28="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H28,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T28,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T28="","PENDENTE",IF($G28="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H28,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T28,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J28" s="13">
@@ -3125,7 +3125,7 @@
         <v/>
       </c>
       <c r="I29" s="12">
-        <f>IF($T29="","PENDENTE",IF($G29="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H29,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T29,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T29="","PENDENTE",IF($G29="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H29,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T29,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J29" s="13">
@@ -3212,7 +3212,7 @@
         <v/>
       </c>
       <c r="I30" s="12">
-        <f>IF($T30="","PENDENTE",IF($G30="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H30,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T30,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T30="","PENDENTE",IF($G30="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H30,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T30,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J30" s="13">
@@ -3299,7 +3299,7 @@
         <v/>
       </c>
       <c r="I31" s="12">
-        <f>IF($T31="","PENDENTE",IF($G31="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H31,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T31,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T31="","PENDENTE",IF($G31="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H31,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T31,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J31" s="13">
@@ -3386,7 +3386,7 @@
         <v/>
       </c>
       <c r="I32" s="12">
-        <f>IF($T32="","PENDENTE",IF($G32="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H32,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T32,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T32="","PENDENTE",IF($G32="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H32,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T32,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J32" s="13">
@@ -3473,7 +3473,7 @@
         <v/>
       </c>
       <c r="I33" s="12">
-        <f>IF($T33="","PENDENTE",IF($G33="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H33,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T33,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T33="","PENDENTE",IF($G33="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H33,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T33,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J33" s="13">
@@ -3560,7 +3560,7 @@
         <v/>
       </c>
       <c r="I34" s="12">
-        <f>IF($T34="","PENDENTE",IF($G34="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H34,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T34,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T34="","PENDENTE",IF($G34="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H34,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T34,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J34" s="13">
@@ -3647,7 +3647,7 @@
         <v/>
       </c>
       <c r="I35" s="12">
-        <f>IF($T35="","PENDENTE",IF($G35="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H35,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T35,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T35="","PENDENTE",IF($G35="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H35,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T35,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J35" s="13">
@@ -3734,7 +3734,7 @@
         <v/>
       </c>
       <c r="I36" s="12">
-        <f>IF($T36="","PENDENTE",IF($G36="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H36,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T36,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T36="","PENDENTE",IF($G36="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H36,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T36,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J36" s="13">
@@ -3821,7 +3821,7 @@
         <v/>
       </c>
       <c r="I37" s="12">
-        <f>IF($T37="","PENDENTE",IF($G37="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H37,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T37,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T37="","PENDENTE",IF($G37="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H37,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T37,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J37" s="13">
@@ -3908,7 +3908,7 @@
         <v/>
       </c>
       <c r="I38" s="12">
-        <f>IF($T38="","PENDENTE",IF($G38="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H38,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T38,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T38="","PENDENTE",IF($G38="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H38,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T38,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J38" s="13">
@@ -3995,7 +3995,7 @@
         <v/>
       </c>
       <c r="I39" s="12">
-        <f>IF($T39="","PENDENTE",IF($G39="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H39,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T39,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T39="","PENDENTE",IF($G39="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H39,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T39,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J39" s="13">
@@ -4082,7 +4082,7 @@
         <v/>
       </c>
       <c r="I40" s="12">
-        <f>IF($T40="","PENDENTE",IF($G40="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H40,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T40,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T40="","PENDENTE",IF($G40="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H40,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T40,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J40" s="13">
@@ -4169,7 +4169,7 @@
         <v/>
       </c>
       <c r="I41" s="12">
-        <f>IF($T41="","PENDENTE",IF($G41="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H41,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T41,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T41="","PENDENTE",IF($G41="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H41,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T41,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J41" s="13">
@@ -4263,7 +4263,7 @@
         <v/>
       </c>
       <c r="I44" s="12">
-        <f>IF($T44="","PENDENTE",IF($G44="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H44,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T44,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T44="","PENDENTE",IF($G44="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H44,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T44,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J44" s="13">
@@ -4350,7 +4350,7 @@
         <v/>
       </c>
       <c r="I45" s="12">
-        <f>IF($T45="","PENDENTE",IF($G45="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H45,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T45,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T45="","PENDENTE",IF($G45="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H45,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T45,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J45" s="13">
@@ -4437,7 +4437,7 @@
         <v/>
       </c>
       <c r="I46" s="12">
-        <f>IF($T46="","PENDENTE",IF($G46="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H46,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T46,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T46="","PENDENTE",IF($G46="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H46,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T46,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J46" s="13">
@@ -4524,7 +4524,7 @@
         <v/>
       </c>
       <c r="I47" s="12">
-        <f>IF($T47="","PENDENTE",IF($G47="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H47,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T47,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T47="","PENDENTE",IF($G47="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H47,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T47,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J47" s="13">
@@ -4611,7 +4611,7 @@
         <v/>
       </c>
       <c r="I48" s="12">
-        <f>IF($T48="","PENDENTE",IF($G48="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H48,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T48,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T48="","PENDENTE",IF($G48="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H48,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T48,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J48" s="13">
@@ -4698,7 +4698,7 @@
         <v/>
       </c>
       <c r="I49" s="12">
-        <f>IF($T49="","PENDENTE",IF($G49="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H49,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T49,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T49="","PENDENTE",IF($G49="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H49,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T49,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J49" s="13">
@@ -4785,7 +4785,7 @@
         <v/>
       </c>
       <c r="I50" s="12">
-        <f>IF($T50="","PENDENTE",IF($G50="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H50,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T50,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T50="","PENDENTE",IF($G50="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H50,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T50,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J50" s="13">
@@ -4872,7 +4872,7 @@
         <v/>
       </c>
       <c r="I51" s="12">
-        <f>IF($T51="","PENDENTE",IF($G51="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H51,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T51,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T51="","PENDENTE",IF($G51="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H51,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T51,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J51" s="13">
@@ -4959,7 +4959,7 @@
         <v/>
       </c>
       <c r="I52" s="12">
-        <f>IF($T52="","PENDENTE",IF($G52="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H52,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T52,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T52="","PENDENTE",IF($G52="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H52,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T52,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J52" s="13">
@@ -5046,7 +5046,7 @@
         <v/>
       </c>
       <c r="I53" s="12">
-        <f>IF($T53="","PENDENTE",IF($G53="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H53,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T53,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T53="","PENDENTE",IF($G53="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H53,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T53,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J53" s="13">
@@ -5133,7 +5133,7 @@
         <v/>
       </c>
       <c r="I54" s="12">
-        <f>IF($T54="","PENDENTE",IF($G54="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H54,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T54,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T54="","PENDENTE",IF($G54="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H54,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T54,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J54" s="13">
@@ -5220,7 +5220,7 @@
         <v/>
       </c>
       <c r="I55" s="12">
-        <f>IF($T55="","PENDENTE",IF($G55="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H55,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T55,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T55="","PENDENTE",IF($G55="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H55,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T55,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J55" s="13">
@@ -5307,7 +5307,7 @@
         <v/>
       </c>
       <c r="I56" s="12">
-        <f>IF($T56="","PENDENTE",IF($G56="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H56,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T56,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T56="","PENDENTE",IF($G56="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H56,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T56,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J56" s="13">
@@ -5394,7 +5394,7 @@
         <v/>
       </c>
       <c r="I57" s="12">
-        <f>IF($T57="","PENDENTE",IF($G57="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H57,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T57,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T57="","PENDENTE",IF($G57="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H57,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T57,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J57" s="13">
@@ -5481,7 +5481,7 @@
         <v/>
       </c>
       <c r="I58" s="12">
-        <f>IF($T58="","PENDENTE",IF($G58="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H58,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T58,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T58="","PENDENTE",IF($G58="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H58,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T58,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J58" s="13">
@@ -5575,7 +5575,7 @@
         <v/>
       </c>
       <c r="I61" s="12">
-        <f>IF($T61="","PENDENTE",IF($G61="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H61,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T61,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T61="","PENDENTE",IF($G61="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H61,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T61,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J61" s="13">
@@ -5662,7 +5662,7 @@
         <v/>
       </c>
       <c r="I62" s="12">
-        <f>IF($T62="","PENDENTE",IF($G62="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H62,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T62,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T62="","PENDENTE",IF($G62="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H62,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T62,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J62" s="13">
@@ -5749,7 +5749,7 @@
         <v/>
       </c>
       <c r="I63" s="12">
-        <f>IF($T63="","PENDENTE",IF($G63="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H63,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T63,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T63="","PENDENTE",IF($G63="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H63,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T63,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J63" s="13">
@@ -5836,7 +5836,7 @@
         <v/>
       </c>
       <c r="I64" s="12">
-        <f>IF($T64="","PENDENTE",IF($G64="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H64,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T64,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T64="","PENDENTE",IF($G64="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H64,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T64,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J64" s="13">
@@ -5923,7 +5923,7 @@
         <v/>
       </c>
       <c r="I65" s="12">
-        <f>IF($T65="","PENDENTE",IF($G65="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H65,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T65,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T65="","PENDENTE",IF($G65="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H65,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T65,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J65" s="13">
@@ -6010,7 +6010,7 @@
         <v/>
       </c>
       <c r="I66" s="12">
-        <f>IF($T66="","PENDENTE",IF($G66="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H66,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T66,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T66="","PENDENTE",IF($G66="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H66,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T66,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J66" s="13">
@@ -6097,7 +6097,7 @@
         <v/>
       </c>
       <c r="I67" s="12">
-        <f>IF($T67="","PENDENTE",IF($G67="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H67,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T67,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T67="","PENDENTE",IF($G67="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H67,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T67,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J67" s="13">
@@ -6184,7 +6184,7 @@
         <v/>
       </c>
       <c r="I68" s="12">
-        <f>IF($T68="","PENDENTE",IF($G68="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H68,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T68,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T68="","PENDENTE",IF($G68="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H68,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T68,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J68" s="13">
@@ -6271,7 +6271,7 @@
         <v/>
       </c>
       <c r="I69" s="12">
-        <f>IF($T69="","PENDENTE",IF($G69="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H69,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T69,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T69="","PENDENTE",IF($G69="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H69,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T69,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J69" s="13">
@@ -6358,7 +6358,7 @@
         <v/>
       </c>
       <c r="I70" s="12">
-        <f>IF($T70="","PENDENTE",IF($G70="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H70,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T70,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T70="","PENDENTE",IF($G70="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H70,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T70,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J70" s="13">
@@ -6445,7 +6445,7 @@
         <v/>
       </c>
       <c r="I71" s="12">
-        <f>IF($T71="","PENDENTE",IF($G71="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H71,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T71,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T71="","PENDENTE",IF($G71="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H71,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T71,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J71" s="13">
@@ -6532,7 +6532,7 @@
         <v/>
       </c>
       <c r="I72" s="12">
-        <f>IF($T72="","PENDENTE",IF($G72="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H72,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T72,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T72="","PENDENTE",IF($G72="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H72,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T72,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J72" s="13">
@@ -6619,7 +6619,7 @@
         <v/>
       </c>
       <c r="I73" s="12">
-        <f>IF($T73="","PENDENTE",IF($G73="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H73,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T73,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T73="","PENDENTE",IF($G73="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H73,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T73,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J73" s="13">
@@ -6706,7 +6706,7 @@
         <v/>
       </c>
       <c r="I74" s="12">
-        <f>IF($T74="","PENDENTE",IF($G74="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H74,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T74,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T74="","PENDENTE",IF($G74="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H74,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T74,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J74" s="13">
@@ -6793,7 +6793,7 @@
         <v/>
       </c>
       <c r="I75" s="12">
-        <f>IF($T75="","PENDENTE",IF($G75="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H75,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T75,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T75="","PENDENTE",IF($G75="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H75,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T75,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J75" s="13">
@@ -6880,7 +6880,7 @@
         <v/>
       </c>
       <c r="I76" s="12">
-        <f>IF($T76="","PENDENTE",IF($G76="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H76,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T76,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T76="","PENDENTE",IF($G76="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H76,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T76,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J76" s="13">
@@ -6967,7 +6967,7 @@
         <v/>
       </c>
       <c r="I77" s="12">
-        <f>IF($T77="","PENDENTE",IF($G77="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H77,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T77,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T77="","PENDENTE",IF($G77="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H77,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T77,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J77" s="13">
@@ -7054,7 +7054,7 @@
         <v/>
       </c>
       <c r="I78" s="12">
-        <f>IF($T78="","PENDENTE",IF($G78="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H78,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T78,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T78="","PENDENTE",IF($G78="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H78,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T78,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J78" s="13">
@@ -7141,7 +7141,7 @@
         <v/>
       </c>
       <c r="I79" s="12">
-        <f>IF($T79="","PENDENTE",IF($G79="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H79,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T79,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T79="","PENDENTE",IF($G79="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H79,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T79,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J79" s="13">
@@ -7235,7 +7235,7 @@
         <v/>
       </c>
       <c r="I82" s="12">
-        <f>IF($T82="","PENDENTE",IF($G82="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H82,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T82,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T82="","PENDENTE",IF($G82="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H82,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T82,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J82" s="13">
@@ -7322,7 +7322,7 @@
         <v/>
       </c>
       <c r="I83" s="12">
-        <f>IF($T83="","PENDENTE",IF($G83="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H83,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T83,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T83="","PENDENTE",IF($G83="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H83,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T83,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J83" s="13">
@@ -7409,7 +7409,7 @@
         <v/>
       </c>
       <c r="I84" s="12">
-        <f>IF($T84="","PENDENTE",IF($G84="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H84,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T84,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T84="","PENDENTE",IF($G84="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H84,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T84,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J84" s="13">
@@ -7496,7 +7496,7 @@
         <v/>
       </c>
       <c r="I85" s="12">
-        <f>IF($T85="","PENDENTE",IF($G85="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H85,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T85,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T85="","PENDENTE",IF($G85="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H85,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T85,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J85" s="13">
@@ -7583,7 +7583,7 @@
         <v/>
       </c>
       <c r="I86" s="12">
-        <f>IF($T86="","PENDENTE",IF($G86="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H86,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T86,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T86="","PENDENTE",IF($G86="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H86,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T86,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J86" s="13">
@@ -7670,7 +7670,7 @@
         <v/>
       </c>
       <c r="I87" s="12">
-        <f>IF($T87="","PENDENTE",IF($G87="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H87,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T87,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T87="","PENDENTE",IF($G87="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H87,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T87,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J87" s="13">
@@ -7757,7 +7757,7 @@
         <v/>
       </c>
       <c r="I88" s="12">
-        <f>IF($T88="","PENDENTE",IF($G88="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H88,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T88,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T88="","PENDENTE",IF($G88="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H88,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T88,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J88" s="13">
@@ -7844,7 +7844,7 @@
         <v/>
       </c>
       <c r="I89" s="12">
-        <f>IF($T89="","PENDENTE",IF($G89="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H89,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T89,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T89="","PENDENTE",IF($G89="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H89,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T89,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J89" s="13">
@@ -7931,7 +7931,7 @@
         <v/>
       </c>
       <c r="I90" s="12">
-        <f>IF($T90="","PENDENTE",IF($G90="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H90,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T90,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T90="","PENDENTE",IF($G90="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H90,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T90,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J90" s="13">
@@ -8018,7 +8018,7 @@
         <v/>
       </c>
       <c r="I91" s="12">
-        <f>IF($T91="","PENDENTE",IF($G91="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H91,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T91,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T91="","PENDENTE",IF($G91="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H91,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T91,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J91" s="13">
@@ -8105,7 +8105,7 @@
         <v/>
       </c>
       <c r="I92" s="12">
-        <f>IF($T92="","PENDENTE",IF($G92="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H92,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T92,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T92="","PENDENTE",IF($G92="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H92,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T92,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J92" s="13">
@@ -8192,7 +8192,7 @@
         <v/>
       </c>
       <c r="I93" s="12">
-        <f>IF($T93="","PENDENTE",IF($G93="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H93,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T93,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T93="","PENDENTE",IF($G93="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H93,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T93,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J93" s="13">
@@ -8279,7 +8279,7 @@
         <v/>
       </c>
       <c r="I94" s="12">
-        <f>IF($T94="","PENDENTE",IF($G94="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H94,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T94,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T94="","PENDENTE",IF($G94="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H94,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T94,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J94" s="13">
@@ -8366,7 +8366,7 @@
         <v/>
       </c>
       <c r="I95" s="12">
-        <f>IF($T95="","PENDENTE",IF($G95="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H95,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T95,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T95="","PENDENTE",IF($G95="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H95,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T95,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J95" s="13">
@@ -8838,7 +8838,7 @@
         <v/>
       </c>
       <c r="I6" s="12">
-        <f>IF($T6="","PENDENTE",IF($G6="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H6,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T6,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T6="","PENDENTE",IF($G6="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H6,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T6,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J6" s="13">
@@ -8921,7 +8921,7 @@
         <v/>
       </c>
       <c r="I7" s="12">
-        <f>IF($T7="","PENDENTE",IF($G7="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H7,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T7,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T7="","PENDENTE",IF($G7="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H7,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T7,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J7" s="13">
@@ -9004,7 +9004,7 @@
         <v/>
       </c>
       <c r="I8" s="12">
-        <f>IF($T8="","PENDENTE",IF($G8="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H8,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T8,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T8="","PENDENTE",IF($G8="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H8,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T8,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J8" s="13">
@@ -9087,7 +9087,7 @@
         <v/>
       </c>
       <c r="I9" s="12">
-        <f>IF($T9="","PENDENTE",IF($G9="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H9,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T9,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T9="","PENDENTE",IF($G9="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H9,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T9,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J9" s="13">
@@ -9170,7 +9170,7 @@
         <v/>
       </c>
       <c r="I10" s="12">
-        <f>IF($T10="","PENDENTE",IF($G10="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H10,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T10,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T10="","PENDENTE",IF($G10="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H10,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T10,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J10" s="13">
@@ -9450,7 +9450,7 @@
         <v/>
       </c>
       <c r="I6" s="12">
-        <f>IF($T6="","PENDENTE",IF($G6="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H6,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T6,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T6="","PENDENTE",IF($G6="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H6,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T6,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J6" s="13">
@@ -9490,7 +9490,11 @@
         <f>IF(OR($M6="",$M6=0),"-",IF($M6&gt;=2*TURNO,"Alta",IF($M6&gt;=TURNO,"Media","Baixa")))</f>
         <v/>
       </c>
-      <c r="T6" s="17" t="inlineStr"/>
+      <c r="T6" s="17" t="inlineStr">
+        <is>
+          <t>CACAU</t>
+        </is>
+      </c>
       <c r="U6" s="8" t="inlineStr">
         <is>
           <t>P1</t>
@@ -9529,7 +9533,7 @@
         <v/>
       </c>
       <c r="I7" s="12">
-        <f>IF($T7="","PENDENTE",IF($G7="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H7,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T7,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T7="","PENDENTE",IF($G7="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H7,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T7,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J7" s="13">
@@ -9569,7 +9573,11 @@
         <f>IF(OR($M7="",$M7=0),"-",IF($M7&gt;=2*TURNO,"Alta",IF($M7&gt;=TURNO,"Media","Baixa")))</f>
         <v/>
       </c>
-      <c r="T7" s="17" t="inlineStr"/>
+      <c r="T7" s="17" t="inlineStr">
+        <is>
+          <t>CACAU</t>
+        </is>
+      </c>
       <c r="U7" s="8" t="inlineStr">
         <is>
           <t>P2</t>
@@ -9608,7 +9616,7 @@
         <v/>
       </c>
       <c r="I8" s="12">
-        <f>IF($T8="","PENDENTE",IF($G8="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H8,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T8,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T8="","PENDENTE",IF($G8="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H8,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T8,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J8" s="13">
@@ -9648,7 +9656,11 @@
         <f>IF(OR($M8="",$M8=0),"-",IF($M8&gt;=2*TURNO,"Alta",IF($M8&gt;=TURNO,"Media","Baixa")))</f>
         <v/>
       </c>
-      <c r="T8" s="17" t="inlineStr"/>
+      <c r="T8" s="17" t="inlineStr">
+        <is>
+          <t>CACAU</t>
+        </is>
+      </c>
       <c r="U8" s="8" t="inlineStr">
         <is>
           <t>P3</t>
@@ -9687,7 +9699,7 @@
         <v/>
       </c>
       <c r="I9" s="12">
-        <f>IF($T9="","PENDENTE",IF($G9="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H9,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T9,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T9="","PENDENTE",IF($G9="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H9,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T9,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J9" s="13">
@@ -9727,7 +9739,11 @@
         <f>IF(OR($M9="",$M9=0),"-",IF($M9&gt;=2*TURNO,"Alta",IF($M9&gt;=TURNO,"Media","Baixa")))</f>
         <v/>
       </c>
-      <c r="T9" s="17" t="inlineStr"/>
+      <c r="T9" s="17" t="inlineStr">
+        <is>
+          <t>CACAU</t>
+        </is>
+      </c>
       <c r="U9" s="8" t="inlineStr">
         <is>
           <t>P25</t>
@@ -9766,7 +9782,7 @@
         <v/>
       </c>
       <c r="I10" s="12">
-        <f>IF($T10="","PENDENTE",IF($G10="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H10,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T10,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T10="","PENDENTE",IF($G10="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H10,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T10,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J10" s="13">
@@ -9806,7 +9822,11 @@
         <f>IF(OR($M10="",$M10=0),"-",IF($M10&gt;=2*TURNO,"Alta",IF($M10&gt;=TURNO,"Media","Baixa")))</f>
         <v/>
       </c>
-      <c r="T10" s="17" t="inlineStr"/>
+      <c r="T10" s="17" t="inlineStr">
+        <is>
+          <t>CACAU</t>
+        </is>
+      </c>
       <c r="U10" s="8" t="inlineStr">
         <is>
           <t>P27</t>
@@ -9845,7 +9865,7 @@
         <v/>
       </c>
       <c r="I11" s="12">
-        <f>IF($T11="","PENDENTE",IF($G11="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H11,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T11,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T11="","PENDENTE",IF($G11="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H11,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T11,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J11" s="13">
@@ -9885,7 +9905,11 @@
         <f>IF(OR($M11="",$M11=0),"-",IF($M11&gt;=2*TURNO,"Alta",IF($M11&gt;=TURNO,"Media","Baixa")))</f>
         <v/>
       </c>
-      <c r="T11" s="17" t="inlineStr"/>
+      <c r="T11" s="17" t="inlineStr">
+        <is>
+          <t>CACAU</t>
+        </is>
+      </c>
       <c r="U11" s="8" t="inlineStr">
         <is>
           <t>P28</t>
@@ -9924,7 +9948,7 @@
         <v/>
       </c>
       <c r="I12" s="12">
-        <f>IF($T12="","PENDENTE",IF($G12="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H12,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T12,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T12="","PENDENTE",IF($G12="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H12,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T12,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J12" s="13">
@@ -9964,7 +9988,11 @@
         <f>IF(OR($M12="",$M12=0),"-",IF($M12&gt;=2*TURNO,"Alta",IF($M12&gt;=TURNO,"Media","Baixa")))</f>
         <v/>
       </c>
-      <c r="T12" s="17" t="inlineStr"/>
+      <c r="T12" s="17" t="inlineStr">
+        <is>
+          <t>CACAU</t>
+        </is>
+      </c>
       <c r="U12" s="8" t="inlineStr">
         <is>
           <t>P29</t>
@@ -10003,7 +10031,7 @@
         <v/>
       </c>
       <c r="I13" s="12">
-        <f>IF($T13="","PENDENTE",IF($G13="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H13,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T13,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T13="","PENDENTE",IF($G13="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H13,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T13,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J13" s="13">
@@ -10043,7 +10071,11 @@
         <f>IF(OR($M13="",$M13=0),"-",IF($M13&gt;=2*TURNO,"Alta",IF($M13&gt;=TURNO,"Media","Baixa")))</f>
         <v/>
       </c>
-      <c r="T13" s="17" t="inlineStr"/>
+      <c r="T13" s="17" t="inlineStr">
+        <is>
+          <t>CACAU</t>
+        </is>
+      </c>
       <c r="U13" s="8" t="inlineStr">
         <is>
           <t>P30</t>
@@ -10082,7 +10114,7 @@
         <v/>
       </c>
       <c r="I14" s="12">
-        <f>IF($T14="","PENDENTE",IF($G14="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H14,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T14,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T14="","PENDENTE",IF($G14="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H14,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T14,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J14" s="13">
@@ -10122,7 +10154,11 @@
         <f>IF(OR($M14="",$M14=0),"-",IF($M14&gt;=2*TURNO,"Alta",IF($M14&gt;=TURNO,"Media","Baixa")))</f>
         <v/>
       </c>
-      <c r="T14" s="17" t="inlineStr"/>
+      <c r="T14" s="17" t="inlineStr">
+        <is>
+          <t>CACAU</t>
+        </is>
+      </c>
       <c r="U14" s="8" t="inlineStr">
         <is>
           <t>P31</t>
@@ -10161,7 +10197,7 @@
         <v/>
       </c>
       <c r="I15" s="12">
-        <f>IF($T15="","PENDENTE",IF($G15="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H15,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T15,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T15="","PENDENTE",IF($G15="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H15,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T15,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J15" s="13">
@@ -10201,7 +10237,11 @@
         <f>IF(OR($M15="",$M15=0),"-",IF($M15&gt;=2*TURNO,"Alta",IF($M15&gt;=TURNO,"Media","Baixa")))</f>
         <v/>
       </c>
-      <c r="T15" s="17" t="inlineStr"/>
+      <c r="T15" s="17" t="inlineStr">
+        <is>
+          <t>CACAU</t>
+        </is>
+      </c>
       <c r="U15" s="8" t="inlineStr">
         <is>
           <t>P32</t>
@@ -10240,7 +10280,7 @@
         <v/>
       </c>
       <c r="I16" s="12">
-        <f>IF($T16="","PENDENTE",IF($G16="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H16,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T16,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T16="","PENDENTE",IF($G16="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H16,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T16,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J16" s="13">
@@ -10280,7 +10320,11 @@
         <f>IF(OR($M16="",$M16=0),"-",IF($M16&gt;=2*TURNO,"Alta",IF($M16&gt;=TURNO,"Media","Baixa")))</f>
         <v/>
       </c>
-      <c r="T16" s="17" t="inlineStr"/>
+      <c r="T16" s="17" t="inlineStr">
+        <is>
+          <t>CACAU</t>
+        </is>
+      </c>
       <c r="U16" s="8" t="inlineStr">
         <is>
           <t>P34</t>
@@ -10319,7 +10363,7 @@
         <v/>
       </c>
       <c r="I17" s="12">
-        <f>IF($T17="","PENDENTE",IF($G17="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H17,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T17,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T17="","PENDENTE",IF($G17="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H17,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T17,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J17" s="13">
@@ -10359,7 +10403,11 @@
         <f>IF(OR($M17="",$M17=0),"-",IF($M17&gt;=2*TURNO,"Alta",IF($M17&gt;=TURNO,"Media","Baixa")))</f>
         <v/>
       </c>
-      <c r="T17" s="17" t="inlineStr"/>
+      <c r="T17" s="17" t="inlineStr">
+        <is>
+          <t>CACAU</t>
+        </is>
+      </c>
       <c r="U17" s="8" t="inlineStr">
         <is>
           <t>P75</t>
@@ -10398,7 +10446,7 @@
         <v/>
       </c>
       <c r="I18" s="12">
-        <f>IF($T18="","PENDENTE",IF($G18="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$I$224,MATCH(MIN(MAX($H18,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T18,CURVAS_KC!$B$4:$I$4,0)),"PENDENTE")))</f>
+        <f>IF($T18="","PENDENTE",IF($G18="","(nao plantado)",IFERROR(INDEX(CURVAS_KC!$B$5:$J$224,MATCH(MIN(MAX($H18,1),220),CURVAS_KC!$A$5:$A$224,0),MATCH($T18,CURVAS_KC!$B$4:$J$4,0)),"PENDENTE")))</f>
         <v/>
       </c>
       <c r="J18" s="13">
@@ -10438,7 +10486,11 @@
         <f>IF(OR($M18="",$M18=0),"-",IF($M18&gt;=2*TURNO,"Alta",IF($M18&gt;=TURNO,"Media","Baixa")))</f>
         <v/>
       </c>
-      <c r="T18" s="17" t="inlineStr"/>
+      <c r="T18" s="17" t="inlineStr">
+        <is>
+          <t>CACAU</t>
+        </is>
+      </c>
       <c r="U18" s="8" t="inlineStr">
         <is>
           <t>P76</t>
@@ -11258,7 +11310,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I224"/>
+  <dimension ref="A1:J224"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -11270,6 +11322,7 @@
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -11332,6 +11385,11 @@
           <t>TABACO</t>
         </is>
       </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>CACAU</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="25" t="n">
@@ -11360,6 +11418,9 @@
       </c>
       <c r="I5" s="26" t="n">
         <v>0.35</v>
+      </c>
+      <c r="J5" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -11390,6 +11451,9 @@
       <c r="I6" s="26" t="n">
         <v>0.35</v>
       </c>
+      <c r="J6" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="25" t="n">
@@ -11419,6 +11483,9 @@
       <c r="I7" s="26" t="n">
         <v>0.35</v>
       </c>
+      <c r="J7" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="25" t="n">
@@ -11448,6 +11515,9 @@
       <c r="I8" s="26" t="n">
         <v>0.35</v>
       </c>
+      <c r="J8" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="25" t="n">
@@ -11477,6 +11547,9 @@
       <c r="I9" s="26" t="n">
         <v>0.35</v>
       </c>
+      <c r="J9" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="25" t="n">
@@ -11506,6 +11579,9 @@
       <c r="I10" s="26" t="n">
         <v>0.35</v>
       </c>
+      <c r="J10" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="25" t="n">
@@ -11535,6 +11611,9 @@
       <c r="I11" s="26" t="n">
         <v>0.35</v>
       </c>
+      <c r="J11" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="25" t="n">
@@ -11564,6 +11643,9 @@
       <c r="I12" s="26" t="n">
         <v>0.35</v>
       </c>
+      <c r="J12" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="25" t="n">
@@ -11593,6 +11675,9 @@
       <c r="I13" s="26" t="n">
         <v>0.35</v>
       </c>
+      <c r="J13" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="25" t="n">
@@ -11622,6 +11707,9 @@
       <c r="I14" s="26" t="n">
         <v>0.35</v>
       </c>
+      <c r="J14" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="25" t="n">
@@ -11649,7 +11737,10 @@
         <v>0.65</v>
       </c>
       <c r="I15" s="26" t="n">
-        <v>0.382</v>
+        <v>0.35</v>
+      </c>
+      <c r="J15" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -11678,7 +11769,10 @@
         <v>0.65</v>
       </c>
       <c r="I16" s="26" t="n">
-        <v>0.414</v>
+        <v>0.35</v>
+      </c>
+      <c r="J16" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -11707,7 +11801,10 @@
         <v>0.65</v>
       </c>
       <c r="I17" s="26" t="n">
-        <v>0.446</v>
+        <v>0.35</v>
+      </c>
+      <c r="J17" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -11736,7 +11833,10 @@
         <v>0.65</v>
       </c>
       <c r="I18" s="26" t="n">
-        <v>0.478</v>
+        <v>0.35</v>
+      </c>
+      <c r="J18" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -11765,7 +11865,10 @@
         <v>0.65</v>
       </c>
       <c r="I19" s="26" t="n">
-        <v>0.51</v>
+        <v>0.35</v>
+      </c>
+      <c r="J19" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -11794,7 +11897,10 @@
         <v>0.654</v>
       </c>
       <c r="I20" s="26" t="n">
-        <v>0.542</v>
+        <v>0.35</v>
+      </c>
+      <c r="J20" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -11823,7 +11929,10 @@
         <v>0.659</v>
       </c>
       <c r="I21" s="26" t="n">
-        <v>0.574</v>
+        <v>0.35</v>
+      </c>
+      <c r="J21" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -11852,7 +11961,10 @@
         <v>0.663</v>
       </c>
       <c r="I22" s="26" t="n">
-        <v>0.606</v>
+        <v>0.35</v>
+      </c>
+      <c r="J22" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -11881,7 +11993,10 @@
         <v>0.668</v>
       </c>
       <c r="I23" s="26" t="n">
-        <v>0.638</v>
+        <v>0.35</v>
+      </c>
+      <c r="J23" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -11910,7 +12025,10 @@
         <v>0.672</v>
       </c>
       <c r="I24" s="26" t="n">
-        <v>0.67</v>
+        <v>0.35</v>
+      </c>
+      <c r="J24" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -11939,7 +12057,10 @@
         <v>0.677</v>
       </c>
       <c r="I25" s="26" t="n">
-        <v>0.702</v>
+        <v>0.377</v>
+      </c>
+      <c r="J25" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -11968,7 +12089,10 @@
         <v>0.681</v>
       </c>
       <c r="I26" s="26" t="n">
-        <v>0.734</v>
+        <v>0.403</v>
+      </c>
+      <c r="J26" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -11997,7 +12121,10 @@
         <v>0.6860000000000001</v>
       </c>
       <c r="I27" s="26" t="n">
-        <v>0.766</v>
+        <v>0.43</v>
+      </c>
+      <c r="J27" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -12026,7 +12153,10 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="I28" s="26" t="n">
-        <v>0.798</v>
+        <v>0.457</v>
+      </c>
+      <c r="J28" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="29">
@@ -12055,7 +12185,10 @@
         <v>0.694</v>
       </c>
       <c r="I29" s="26" t="n">
-        <v>0.83</v>
+        <v>0.483</v>
+      </c>
+      <c r="J29" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -12084,7 +12217,10 @@
         <v>0.699</v>
       </c>
       <c r="I30" s="26" t="n">
-        <v>0.862</v>
+        <v>0.51</v>
+      </c>
+      <c r="J30" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -12113,7 +12249,10 @@
         <v>0.703</v>
       </c>
       <c r="I31" s="26" t="n">
-        <v>0.894</v>
+        <v>0.537</v>
+      </c>
+      <c r="J31" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -12142,7 +12281,10 @@
         <v>0.708</v>
       </c>
       <c r="I32" s="26" t="n">
-        <v>0.926</v>
+        <v>0.5629999999999999</v>
+      </c>
+      <c r="J32" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -12171,7 +12313,10 @@
         <v>0.712</v>
       </c>
       <c r="I33" s="26" t="n">
-        <v>0.958</v>
+        <v>0.59</v>
+      </c>
+      <c r="J33" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -12200,7 +12345,10 @@
         <v>0.717</v>
       </c>
       <c r="I34" s="26" t="n">
-        <v>0.99</v>
+        <v>0.617</v>
+      </c>
+      <c r="J34" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -12229,7 +12377,10 @@
         <v>0.721</v>
       </c>
       <c r="I35" s="26" t="n">
-        <v>1.022</v>
+        <v>0.643</v>
+      </c>
+      <c r="J35" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -12258,7 +12409,10 @@
         <v>0.726</v>
       </c>
       <c r="I36" s="26" t="n">
-        <v>1.054</v>
+        <v>0.67</v>
+      </c>
+      <c r="J36" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -12287,7 +12441,10 @@
         <v>0.73</v>
       </c>
       <c r="I37" s="26" t="n">
-        <v>1.086</v>
+        <v>0.697</v>
+      </c>
+      <c r="J37" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -12316,7 +12473,10 @@
         <v>0.734</v>
       </c>
       <c r="I38" s="26" t="n">
-        <v>1.118</v>
+        <v>0.723</v>
+      </c>
+      <c r="J38" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -12345,7 +12505,10 @@
         <v>0.739</v>
       </c>
       <c r="I39" s="26" t="n">
-        <v>1.15</v>
+        <v>0.75</v>
+      </c>
+      <c r="J39" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -12374,7 +12537,10 @@
         <v>0.743</v>
       </c>
       <c r="I40" s="26" t="n">
-        <v>1.15</v>
+        <v>0.777</v>
+      </c>
+      <c r="J40" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -12403,7 +12569,10 @@
         <v>0.748</v>
       </c>
       <c r="I41" s="26" t="n">
-        <v>1.15</v>
+        <v>0.803</v>
+      </c>
+      <c r="J41" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="42">
@@ -12432,7 +12601,10 @@
         <v>0.752</v>
       </c>
       <c r="I42" s="26" t="n">
-        <v>1.15</v>
+        <v>0.83</v>
+      </c>
+      <c r="J42" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -12461,7 +12633,10 @@
         <v>0.757</v>
       </c>
       <c r="I43" s="26" t="n">
-        <v>1.15</v>
+        <v>0.857</v>
+      </c>
+      <c r="J43" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -12490,7 +12665,10 @@
         <v>0.761</v>
       </c>
       <c r="I44" s="26" t="n">
-        <v>1.15</v>
+        <v>0.883</v>
+      </c>
+      <c r="J44" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -12519,7 +12697,10 @@
         <v>0.766</v>
       </c>
       <c r="I45" s="26" t="n">
-        <v>1.15</v>
+        <v>0.91</v>
+      </c>
+      <c r="J45" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -12548,7 +12729,10 @@
         <v>0.77</v>
       </c>
       <c r="I46" s="26" t="n">
-        <v>1.15</v>
+        <v>0.9370000000000001</v>
+      </c>
+      <c r="J46" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -12577,7 +12761,10 @@
         <v>0.774</v>
       </c>
       <c r="I47" s="26" t="n">
-        <v>1.15</v>
+        <v>0.963</v>
+      </c>
+      <c r="J47" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -12606,7 +12793,10 @@
         <v>0.779</v>
       </c>
       <c r="I48" s="26" t="n">
-        <v>1.15</v>
+        <v>0.99</v>
+      </c>
+      <c r="J48" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="49">
@@ -12635,7 +12825,10 @@
         <v>0.783</v>
       </c>
       <c r="I49" s="26" t="n">
-        <v>1.15</v>
+        <v>1.017</v>
+      </c>
+      <c r="J49" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -12664,7 +12857,10 @@
         <v>0.788</v>
       </c>
       <c r="I50" s="26" t="n">
-        <v>1.15</v>
+        <v>1.043</v>
+      </c>
+      <c r="J50" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -12693,7 +12889,10 @@
         <v>0.792</v>
       </c>
       <c r="I51" s="26" t="n">
-        <v>1.15</v>
+        <v>1.07</v>
+      </c>
+      <c r="J51" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="52">
@@ -12722,7 +12921,10 @@
         <v>0.797</v>
       </c>
       <c r="I52" s="26" t="n">
-        <v>1.15</v>
+        <v>1.097</v>
+      </c>
+      <c r="J52" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="53">
@@ -12751,7 +12953,10 @@
         <v>0.801</v>
       </c>
       <c r="I53" s="26" t="n">
-        <v>1.15</v>
+        <v>1.123</v>
+      </c>
+      <c r="J53" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="54">
@@ -12782,6 +12987,9 @@
       <c r="I54" s="26" t="n">
         <v>1.15</v>
       </c>
+      <c r="J54" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="25" t="n">
@@ -12811,6 +13019,9 @@
       <c r="I55" s="26" t="n">
         <v>1.15</v>
       </c>
+      <c r="J55" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="25" t="n">
@@ -12840,6 +13051,9 @@
       <c r="I56" s="26" t="n">
         <v>1.15</v>
       </c>
+      <c r="J56" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="25" t="n">
@@ -12869,6 +13083,9 @@
       <c r="I57" s="26" t="n">
         <v>1.15</v>
       </c>
+      <c r="J57" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="25" t="n">
@@ -12898,6 +13115,9 @@
       <c r="I58" s="26" t="n">
         <v>1.15</v>
       </c>
+      <c r="J58" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="25" t="n">
@@ -12927,6 +13147,9 @@
       <c r="I59" s="26" t="n">
         <v>1.15</v>
       </c>
+      <c r="J59" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="25" t="n">
@@ -12956,6 +13179,9 @@
       <c r="I60" s="26" t="n">
         <v>1.15</v>
       </c>
+      <c r="J60" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="25" t="n">
@@ -12985,6 +13211,9 @@
       <c r="I61" s="26" t="n">
         <v>1.15</v>
       </c>
+      <c r="J61" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="25" t="n">
@@ -13014,6 +13243,9 @@
       <c r="I62" s="26" t="n">
         <v>1.15</v>
       </c>
+      <c r="J62" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="25" t="n">
@@ -13043,6 +13275,9 @@
       <c r="I63" s="26" t="n">
         <v>1.15</v>
       </c>
+      <c r="J63" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="25" t="n">
@@ -13072,6 +13307,9 @@
       <c r="I64" s="26" t="n">
         <v>1.15</v>
       </c>
+      <c r="J64" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="25" t="n">
@@ -13101,6 +13339,9 @@
       <c r="I65" s="26" t="n">
         <v>1.15</v>
       </c>
+      <c r="J65" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="25" t="n">
@@ -13130,6 +13371,9 @@
       <c r="I66" s="26" t="n">
         <v>1.15</v>
       </c>
+      <c r="J66" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="25" t="n">
@@ -13159,6 +13403,9 @@
       <c r="I67" s="26" t="n">
         <v>1.15</v>
       </c>
+      <c r="J67" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="25" t="n">
@@ -13188,6 +13435,9 @@
       <c r="I68" s="26" t="n">
         <v>1.15</v>
       </c>
+      <c r="J68" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="25" t="n">
@@ -13217,6 +13467,9 @@
       <c r="I69" s="26" t="n">
         <v>1.15</v>
       </c>
+      <c r="J69" s="26" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="25" t="n">
@@ -13244,7 +13497,10 @@
         <v>0.925</v>
       </c>
       <c r="I70" s="26" t="n">
-        <v>1.136</v>
+        <v>1.15</v>
+      </c>
+      <c r="J70" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="71">
@@ -13273,7 +13529,10 @@
         <v>0.9379999999999999</v>
       </c>
       <c r="I71" s="26" t="n">
-        <v>1.122</v>
+        <v>1.15</v>
+      </c>
+      <c r="J71" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="72">
@@ -13302,7 +13561,10 @@
         <v>0.95</v>
       </c>
       <c r="I72" s="26" t="n">
-        <v>1.108</v>
+        <v>1.15</v>
+      </c>
+      <c r="J72" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="73">
@@ -13331,7 +13593,10 @@
         <v>0.963</v>
       </c>
       <c r="I73" s="26" t="n">
-        <v>1.094</v>
+        <v>1.15</v>
+      </c>
+      <c r="J73" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="74">
@@ -13360,7 +13625,10 @@
         <v>0.975</v>
       </c>
       <c r="I74" s="26" t="n">
-        <v>1.08</v>
+        <v>1.15</v>
+      </c>
+      <c r="J74" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="75">
@@ -13389,7 +13657,10 @@
         <v>0.988</v>
       </c>
       <c r="I75" s="26" t="n">
-        <v>1.066</v>
+        <v>1.15</v>
+      </c>
+      <c r="J75" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="76">
@@ -13418,7 +13689,10 @@
         <v>1</v>
       </c>
       <c r="I76" s="26" t="n">
-        <v>1.052</v>
+        <v>1.15</v>
+      </c>
+      <c r="J76" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="77">
@@ -13447,7 +13721,10 @@
         <v>1.012</v>
       </c>
       <c r="I77" s="26" t="n">
-        <v>1.038</v>
+        <v>1.15</v>
+      </c>
+      <c r="J77" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="78">
@@ -13476,7 +13753,10 @@
         <v>1.025</v>
       </c>
       <c r="I78" s="26" t="n">
-        <v>1.024</v>
+        <v>1.15</v>
+      </c>
+      <c r="J78" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="79">
@@ -13505,7 +13785,10 @@
         <v>1.038</v>
       </c>
       <c r="I79" s="26" t="n">
-        <v>1.01</v>
+        <v>1.15</v>
+      </c>
+      <c r="J79" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="80">
@@ -13534,7 +13817,10 @@
         <v>1.05</v>
       </c>
       <c r="I80" s="26" t="n">
-        <v>0.996</v>
+        <v>1.15</v>
+      </c>
+      <c r="J80" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="81">
@@ -13563,7 +13849,10 @@
         <v>1.062</v>
       </c>
       <c r="I81" s="26" t="n">
-        <v>0.982</v>
+        <v>1.15</v>
+      </c>
+      <c r="J81" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="82">
@@ -13592,7 +13881,10 @@
         <v>1.075</v>
       </c>
       <c r="I82" s="26" t="n">
-        <v>0.968</v>
+        <v>1.15</v>
+      </c>
+      <c r="J82" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="83">
@@ -13621,7 +13913,10 @@
         <v>1.088</v>
       </c>
       <c r="I83" s="26" t="n">
-        <v>0.954</v>
+        <v>1.15</v>
+      </c>
+      <c r="J83" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="84">
@@ -13650,7 +13945,10 @@
         <v>1.1</v>
       </c>
       <c r="I84" s="26" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.15</v>
+      </c>
+      <c r="J84" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="85">
@@ -13679,7 +13977,10 @@
         <v>1.1</v>
       </c>
       <c r="I85" s="26" t="n">
-        <v>0.926</v>
+        <v>1.142</v>
+      </c>
+      <c r="J85" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="86">
@@ -13708,7 +14009,10 @@
         <v>1.1</v>
       </c>
       <c r="I86" s="26" t="n">
-        <v>0.912</v>
+        <v>1.133</v>
+      </c>
+      <c r="J86" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="87">
@@ -13737,7 +14041,10 @@
         <v>1.1</v>
       </c>
       <c r="I87" s="26" t="n">
-        <v>0.898</v>
+        <v>1.125</v>
+      </c>
+      <c r="J87" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="88">
@@ -13766,7 +14073,10 @@
         <v>1.1</v>
       </c>
       <c r="I88" s="26" t="n">
-        <v>0.884</v>
+        <v>1.117</v>
+      </c>
+      <c r="J88" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="89">
@@ -13795,7 +14105,10 @@
         <v>1.1</v>
       </c>
       <c r="I89" s="26" t="n">
-        <v>0.87</v>
+        <v>1.108</v>
+      </c>
+      <c r="J89" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="90">
@@ -13824,7 +14137,10 @@
         <v>1.1</v>
       </c>
       <c r="I90" s="26" t="n">
-        <v>0.856</v>
+        <v>1.1</v>
+      </c>
+      <c r="J90" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="91">
@@ -13853,7 +14169,10 @@
         <v>1.1</v>
       </c>
       <c r="I91" s="26" t="n">
-        <v>0.842</v>
+        <v>1.092</v>
+      </c>
+      <c r="J91" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="92">
@@ -13882,7 +14201,10 @@
         <v>1.1</v>
       </c>
       <c r="I92" s="26" t="n">
-        <v>0.828</v>
+        <v>1.083</v>
+      </c>
+      <c r="J92" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="93">
@@ -13911,7 +14233,10 @@
         <v>1.1</v>
       </c>
       <c r="I93" s="26" t="n">
-        <v>0.8139999999999999</v>
+        <v>1.075</v>
+      </c>
+      <c r="J93" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="94">
@@ -13940,7 +14265,10 @@
         <v>1.1</v>
       </c>
       <c r="I94" s="26" t="n">
-        <v>0.8</v>
+        <v>1.067</v>
+      </c>
+      <c r="J94" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="95">
@@ -13969,7 +14297,10 @@
         <v>1.1</v>
       </c>
       <c r="I95" s="26" t="n">
-        <v>0.8</v>
+        <v>1.058</v>
+      </c>
+      <c r="J95" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="96">
@@ -13998,7 +14329,10 @@
         <v>1.1</v>
       </c>
       <c r="I96" s="26" t="n">
-        <v>0.8</v>
+        <v>1.05</v>
+      </c>
+      <c r="J96" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="97">
@@ -14027,7 +14361,10 @@
         <v>1.1</v>
       </c>
       <c r="I97" s="26" t="n">
-        <v>0.8</v>
+        <v>1.042</v>
+      </c>
+      <c r="J97" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="98">
@@ -14056,7 +14393,10 @@
         <v>1.1</v>
       </c>
       <c r="I98" s="26" t="n">
-        <v>0.8</v>
+        <v>1.033</v>
+      </c>
+      <c r="J98" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="99">
@@ -14085,7 +14425,10 @@
         <v>1.1</v>
       </c>
       <c r="I99" s="26" t="n">
-        <v>0.8</v>
+        <v>1.025</v>
+      </c>
+      <c r="J99" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="100">
@@ -14114,7 +14457,10 @@
         <v>1.1</v>
       </c>
       <c r="I100" s="26" t="n">
-        <v>0.8</v>
+        <v>1.017</v>
+      </c>
+      <c r="J100" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="101">
@@ -14143,7 +14489,10 @@
         <v>1.1</v>
       </c>
       <c r="I101" s="26" t="n">
-        <v>0.8</v>
+        <v>1.008</v>
+      </c>
+      <c r="J101" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="102">
@@ -14172,7 +14521,10 @@
         <v>1.1</v>
       </c>
       <c r="I102" s="26" t="n">
-        <v>0.8</v>
+        <v>1</v>
+      </c>
+      <c r="J102" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="103">
@@ -14201,7 +14553,10 @@
         <v>1.1</v>
       </c>
       <c r="I103" s="26" t="n">
-        <v>0.8</v>
+        <v>0.992</v>
+      </c>
+      <c r="J103" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="104">
@@ -14230,7 +14585,10 @@
         <v>1.1</v>
       </c>
       <c r="I104" s="26" t="n">
-        <v>0.8</v>
+        <v>0.983</v>
+      </c>
+      <c r="J104" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="105">
@@ -14259,7 +14617,10 @@
         <v>1.1</v>
       </c>
       <c r="I105" s="26" t="n">
-        <v>0.8</v>
+        <v>0.975</v>
+      </c>
+      <c r="J105" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="106">
@@ -14288,7 +14649,10 @@
         <v>1.1</v>
       </c>
       <c r="I106" s="26" t="n">
-        <v>0.8</v>
+        <v>0.967</v>
+      </c>
+      <c r="J106" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="107">
@@ -14317,7 +14681,10 @@
         <v>1.1</v>
       </c>
       <c r="I107" s="26" t="n">
-        <v>0.8</v>
+        <v>0.958</v>
+      </c>
+      <c r="J107" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="108">
@@ -14346,7 +14713,10 @@
         <v>1.1</v>
       </c>
       <c r="I108" s="26" t="n">
-        <v>0.8</v>
+        <v>0.95</v>
+      </c>
+      <c r="J108" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="109">
@@ -14375,7 +14745,10 @@
         <v>1.1</v>
       </c>
       <c r="I109" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9419999999999999</v>
+      </c>
+      <c r="J109" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="110">
@@ -14404,7 +14777,10 @@
         <v>1.08</v>
       </c>
       <c r="I110" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9330000000000001</v>
+      </c>
+      <c r="J110" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="111">
@@ -14433,7 +14809,10 @@
         <v>1.06</v>
       </c>
       <c r="I111" s="26" t="n">
-        <v>0.8</v>
+        <v>0.925</v>
+      </c>
+      <c r="J111" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="112">
@@ -14462,7 +14841,10 @@
         <v>1.04</v>
       </c>
       <c r="I112" s="26" t="n">
-        <v>0.8</v>
+        <v>0.917</v>
+      </c>
+      <c r="J112" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="113">
@@ -14491,7 +14873,10 @@
         <v>1.02</v>
       </c>
       <c r="I113" s="26" t="n">
-        <v>0.8</v>
+        <v>0.908</v>
+      </c>
+      <c r="J113" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="114">
@@ -14520,7 +14905,10 @@
         <v>1</v>
       </c>
       <c r="I114" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J114" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="115">
@@ -14549,7 +14937,10 @@
         <v>0.98</v>
       </c>
       <c r="I115" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J115" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="116">
@@ -14578,7 +14969,10 @@
         <v>0.96</v>
       </c>
       <c r="I116" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J116" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="117">
@@ -14607,7 +15001,10 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="I117" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J117" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="118">
@@ -14636,7 +15033,10 @@
         <v>0.92</v>
       </c>
       <c r="I118" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J118" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="119">
@@ -14665,7 +15065,10 @@
         <v>0.9</v>
       </c>
       <c r="I119" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J119" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="120">
@@ -14694,7 +15097,10 @@
         <v>0.88</v>
       </c>
       <c r="I120" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J120" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="121">
@@ -14723,7 +15129,10 @@
         <v>0.86</v>
       </c>
       <c r="I121" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J121" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="122">
@@ -14752,7 +15161,10 @@
         <v>0.84</v>
       </c>
       <c r="I122" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J122" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="123">
@@ -14781,7 +15193,10 @@
         <v>0.82</v>
       </c>
       <c r="I123" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J123" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="124">
@@ -14810,7 +15225,10 @@
         <v>0.8</v>
       </c>
       <c r="I124" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J124" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="125">
@@ -14839,7 +15257,10 @@
         <v>0.78</v>
       </c>
       <c r="I125" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J125" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="126">
@@ -14868,7 +15289,10 @@
         <v>0.76</v>
       </c>
       <c r="I126" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J126" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="127">
@@ -14897,7 +15321,10 @@
         <v>0.74</v>
       </c>
       <c r="I127" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J127" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="128">
@@ -14926,7 +15353,10 @@
         <v>0.72</v>
       </c>
       <c r="I128" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J128" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="129">
@@ -14955,7 +15385,10 @@
         <v>0.7</v>
       </c>
       <c r="I129" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J129" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="130">
@@ -14984,7 +15417,10 @@
         <v>0.68</v>
       </c>
       <c r="I130" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J130" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="131">
@@ -15013,7 +15449,10 @@
         <v>0.66</v>
       </c>
       <c r="I131" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J131" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="132">
@@ -15042,7 +15481,10 @@
         <v>0.64</v>
       </c>
       <c r="I132" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J132" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="133">
@@ -15071,7 +15513,10 @@
         <v>0.62</v>
       </c>
       <c r="I133" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J133" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="134">
@@ -15100,7 +15545,10 @@
         <v>0.6</v>
       </c>
       <c r="I134" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J134" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="135">
@@ -15129,7 +15577,10 @@
         <v>0.593</v>
       </c>
       <c r="I135" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J135" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="136">
@@ -15158,7 +15609,10 @@
         <v>0.587</v>
       </c>
       <c r="I136" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J136" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="137">
@@ -15187,7 +15641,10 @@
         <v>0.58</v>
       </c>
       <c r="I137" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J137" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="138">
@@ -15216,7 +15673,10 @@
         <v>0.573</v>
       </c>
       <c r="I138" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J138" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="139">
@@ -15245,7 +15705,10 @@
         <v>0.5669999999999999</v>
       </c>
       <c r="I139" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J139" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="140">
@@ -15274,7 +15737,10 @@
         <v>0.5600000000000001</v>
       </c>
       <c r="I140" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J140" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="141">
@@ -15303,7 +15769,10 @@
         <v>0.553</v>
       </c>
       <c r="I141" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J141" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="142">
@@ -15332,7 +15801,10 @@
         <v>0.547</v>
       </c>
       <c r="I142" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J142" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="143">
@@ -15361,7 +15833,10 @@
         <v>0.54</v>
       </c>
       <c r="I143" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J143" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="144">
@@ -15390,7 +15865,10 @@
         <v>0.533</v>
       </c>
       <c r="I144" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J144" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="145">
@@ -15419,7 +15897,10 @@
         <v>0.527</v>
       </c>
       <c r="I145" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J145" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="146">
@@ -15448,7 +15929,10 @@
         <v>0.52</v>
       </c>
       <c r="I146" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J146" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="147">
@@ -15477,7 +15961,10 @@
         <v>0.513</v>
       </c>
       <c r="I147" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J147" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="148">
@@ -15506,7 +15993,10 @@
         <v>0.507</v>
       </c>
       <c r="I148" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J148" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="149">
@@ -15535,7 +16025,10 @@
         <v>0.5</v>
       </c>
       <c r="I149" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J149" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="150">
@@ -15564,7 +16057,10 @@
         <v>0.493</v>
       </c>
       <c r="I150" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J150" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="151">
@@ -15593,7 +16089,10 @@
         <v>0.487</v>
       </c>
       <c r="I151" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J151" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="152">
@@ -15622,7 +16121,10 @@
         <v>0.48</v>
       </c>
       <c r="I152" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J152" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="153">
@@ -15651,7 +16153,10 @@
         <v>0.473</v>
       </c>
       <c r="I153" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J153" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="154">
@@ -15680,7 +16185,10 @@
         <v>0.467</v>
       </c>
       <c r="I154" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J154" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="155">
@@ -15709,7 +16217,10 @@
         <v>0.46</v>
       </c>
       <c r="I155" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J155" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="156">
@@ -15738,7 +16249,10 @@
         <v>0.453</v>
       </c>
       <c r="I156" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J156" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="157">
@@ -15767,7 +16281,10 @@
         <v>0.447</v>
       </c>
       <c r="I157" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J157" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="158">
@@ -15796,7 +16313,10 @@
         <v>0.44</v>
       </c>
       <c r="I158" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J158" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="159">
@@ -15825,7 +16345,10 @@
         <v>0.433</v>
       </c>
       <c r="I159" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J159" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="160">
@@ -15854,7 +16377,10 @@
         <v>0.427</v>
       </c>
       <c r="I160" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J160" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="161">
@@ -15883,7 +16409,10 @@
         <v>0.42</v>
       </c>
       <c r="I161" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J161" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="162">
@@ -15912,7 +16441,10 @@
         <v>0.413</v>
       </c>
       <c r="I162" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J162" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="163">
@@ -15941,7 +16473,10 @@
         <v>0.407</v>
       </c>
       <c r="I163" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J163" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="164">
@@ -15970,7 +16505,10 @@
         <v>0.4</v>
       </c>
       <c r="I164" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J164" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="165">
@@ -15999,7 +16537,10 @@
         <v>0.4</v>
       </c>
       <c r="I165" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J165" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="166">
@@ -16028,7 +16569,10 @@
         <v>0.4</v>
       </c>
       <c r="I166" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J166" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="167">
@@ -16057,7 +16601,10 @@
         <v>0.4</v>
       </c>
       <c r="I167" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J167" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="168">
@@ -16086,7 +16633,10 @@
         <v>0.4</v>
       </c>
       <c r="I168" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J168" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="169">
@@ -16115,7 +16665,10 @@
         <v>0.4</v>
       </c>
       <c r="I169" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J169" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="170">
@@ -16144,7 +16697,10 @@
         <v>0.4</v>
       </c>
       <c r="I170" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J170" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="171">
@@ -16173,7 +16729,10 @@
         <v>0.4</v>
       </c>
       <c r="I171" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J171" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="172">
@@ -16202,7 +16761,10 @@
         <v>0.4</v>
       </c>
       <c r="I172" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J172" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="173">
@@ -16231,7 +16793,10 @@
         <v>0.4</v>
       </c>
       <c r="I173" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J173" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="174">
@@ -16260,7 +16825,10 @@
         <v>0.4</v>
       </c>
       <c r="I174" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J174" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="175">
@@ -16289,7 +16857,10 @@
         <v>0.4</v>
       </c>
       <c r="I175" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J175" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="176">
@@ -16318,7 +16889,10 @@
         <v>0.4</v>
       </c>
       <c r="I176" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J176" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="177">
@@ -16347,7 +16921,10 @@
         <v>0.4</v>
       </c>
       <c r="I177" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J177" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="178">
@@ -16376,7 +16953,10 @@
         <v>0.4</v>
       </c>
       <c r="I178" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J178" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="179">
@@ -16405,7 +16985,10 @@
         <v>0.4</v>
       </c>
       <c r="I179" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J179" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="180">
@@ -16434,7 +17017,10 @@
         <v>0.4</v>
       </c>
       <c r="I180" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J180" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="181">
@@ -16463,7 +17049,10 @@
         <v>0.4</v>
       </c>
       <c r="I181" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J181" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="182">
@@ -16492,7 +17081,10 @@
         <v>0.4</v>
       </c>
       <c r="I182" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J182" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="183">
@@ -16521,7 +17113,10 @@
         <v>0.4</v>
       </c>
       <c r="I183" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J183" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="184">
@@ -16550,7 +17145,10 @@
         <v>0.4</v>
       </c>
       <c r="I184" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J184" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="185">
@@ -16579,7 +17177,10 @@
         <v>0.4</v>
       </c>
       <c r="I185" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J185" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="186">
@@ -16608,7 +17209,10 @@
         <v>0.4</v>
       </c>
       <c r="I186" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J186" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="187">
@@ -16637,7 +17241,10 @@
         <v>0.4</v>
       </c>
       <c r="I187" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J187" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="188">
@@ -16666,7 +17273,10 @@
         <v>0.4</v>
       </c>
       <c r="I188" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J188" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="189">
@@ -16695,7 +17305,10 @@
         <v>0.4</v>
       </c>
       <c r="I189" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J189" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="190">
@@ -16724,7 +17337,10 @@
         <v>0.4</v>
       </c>
       <c r="I190" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J190" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="191">
@@ -16753,7 +17369,10 @@
         <v>0.4</v>
       </c>
       <c r="I191" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J191" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="192">
@@ -16782,7 +17401,10 @@
         <v>0.4</v>
       </c>
       <c r="I192" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J192" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="193">
@@ -16811,7 +17433,10 @@
         <v>0.4</v>
       </c>
       <c r="I193" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J193" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="194">
@@ -16840,7 +17465,10 @@
         <v>0.4</v>
       </c>
       <c r="I194" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J194" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="195">
@@ -16869,7 +17497,10 @@
         <v>0.4</v>
       </c>
       <c r="I195" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J195" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="196">
@@ -16898,7 +17529,10 @@
         <v>0.4</v>
       </c>
       <c r="I196" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J196" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="197">
@@ -16927,7 +17561,10 @@
         <v>0.4</v>
       </c>
       <c r="I197" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J197" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="198">
@@ -16956,7 +17593,10 @@
         <v>0.4</v>
       </c>
       <c r="I198" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J198" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="199">
@@ -16985,7 +17625,10 @@
         <v>0.4</v>
       </c>
       <c r="I199" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J199" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="200">
@@ -17014,7 +17657,10 @@
         <v>0.4</v>
       </c>
       <c r="I200" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J200" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="201">
@@ -17043,7 +17689,10 @@
         <v>0.4</v>
       </c>
       <c r="I201" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J201" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="202">
@@ -17072,7 +17721,10 @@
         <v>0.4</v>
       </c>
       <c r="I202" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J202" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="203">
@@ -17101,7 +17753,10 @@
         <v>0.4</v>
       </c>
       <c r="I203" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J203" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="204">
@@ -17130,7 +17785,10 @@
         <v>0.4</v>
       </c>
       <c r="I204" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J204" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="205">
@@ -17159,7 +17817,10 @@
         <v>0.4</v>
       </c>
       <c r="I205" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J205" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="206">
@@ -17188,7 +17849,10 @@
         <v>0.4</v>
       </c>
       <c r="I206" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J206" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="207">
@@ -17217,7 +17881,10 @@
         <v>0.4</v>
       </c>
       <c r="I207" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J207" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="208">
@@ -17246,7 +17913,10 @@
         <v>0.4</v>
       </c>
       <c r="I208" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J208" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="209">
@@ -17275,7 +17945,10 @@
         <v>0.4</v>
       </c>
       <c r="I209" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J209" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="210">
@@ -17304,7 +17977,10 @@
         <v>0.4</v>
       </c>
       <c r="I210" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J210" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="211">
@@ -17333,7 +18009,10 @@
         <v>0.4</v>
       </c>
       <c r="I211" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J211" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="212">
@@ -17362,7 +18041,10 @@
         <v>0.4</v>
       </c>
       <c r="I212" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J212" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="213">
@@ -17391,7 +18073,10 @@
         <v>0.4</v>
       </c>
       <c r="I213" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J213" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="214">
@@ -17420,7 +18105,10 @@
         <v>0.4</v>
       </c>
       <c r="I214" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J214" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="215">
@@ -17449,7 +18137,10 @@
         <v>0.4</v>
       </c>
       <c r="I215" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J215" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="216">
@@ -17478,7 +18169,10 @@
         <v>0.4</v>
       </c>
       <c r="I216" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J216" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="217">
@@ -17507,7 +18201,10 @@
         <v>0.4</v>
       </c>
       <c r="I217" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J217" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="218">
@@ -17536,7 +18233,10 @@
         <v>0.4</v>
       </c>
       <c r="I218" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J218" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="219">
@@ -17565,7 +18265,10 @@
         <v>0.4</v>
       </c>
       <c r="I219" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J219" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="220">
@@ -17594,7 +18297,10 @@
         <v>0.4</v>
       </c>
       <c r="I220" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J220" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="221">
@@ -17623,7 +18329,10 @@
         <v>0.4</v>
       </c>
       <c r="I221" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J221" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="222">
@@ -17652,7 +18361,10 @@
         <v>0.4</v>
       </c>
       <c r="I222" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J222" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="223">
@@ -17681,7 +18393,10 @@
         <v>0.4</v>
       </c>
       <c r="I223" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J223" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="224">
@@ -17710,7 +18425,10 @@
         <v>0.4</v>
       </c>
       <c r="I224" s="26" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="J224" s="26" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cacau e tabaco com Kc da literatura FAO-56 Tabela 12 (v8.1)
- Cacau (FAO-56 Tabela 12 - cocoa): Kc_ini 0,90 / Kc_mid 1,00 / Kc_end 1,00
  (antes 1,00 fixo; agora inicia em 0,90 para cacau jovem/estabelecimento)
- Tabaco (FAO-56 Tabela 12): Kc_ini 0,35 / Kc_mid 1,10 / Kc_end 0,90
  (meio ajustado de 1,15 para 1,10, valor canonico da tabela)
- Fonte citada no cabecalho da aba CURVAS_KC

Validado: zero erros. Recalculo ao abrir.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019ytrvvbkWKcC1Fp4Ydm9J6
</commit_message>
<xml_diff>
--- a/Manejo_Irrigacao_Karitel_RDM.xlsx
+++ b/Manejo_Irrigacao_Karitel_RDM.xlsx
@@ -29722,7 +29722,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Algodao: arquivo. Soja/milho: por fase. Tabaco/cacau: literatura FAO-56.</t>
+          <t>Fonte: FAO-56 Tabela 12. Soja 0,40/1,15/0,50; Algodao 0,35/1,20/0,60; Milho 0,30/1,20/0,60; Tabaco 0,35/1,10/0,90; Cacau 0,90/1,00/1,00.</t>
         </is>
       </c>
     </row>
@@ -29807,7 +29807,7 @@
         <v>0.35</v>
       </c>
       <c r="J5" s="33" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="6">
@@ -29839,7 +29839,7 @@
         <v>0.35</v>
       </c>
       <c r="J6" s="33" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="7">
@@ -29871,7 +29871,7 @@
         <v>0.35</v>
       </c>
       <c r="J7" s="33" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="8">
@@ -29903,7 +29903,7 @@
         <v>0.35</v>
       </c>
       <c r="J8" s="33" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="9">
@@ -29935,7 +29935,7 @@
         <v>0.35</v>
       </c>
       <c r="J9" s="33" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="10">
@@ -29967,7 +29967,7 @@
         <v>0.35</v>
       </c>
       <c r="J10" s="33" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="11">
@@ -29999,7 +29999,7 @@
         <v>0.35</v>
       </c>
       <c r="J11" s="33" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="12">
@@ -30031,7 +30031,7 @@
         <v>0.35</v>
       </c>
       <c r="J12" s="33" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="13">
@@ -30063,7 +30063,7 @@
         <v>0.35</v>
       </c>
       <c r="J13" s="33" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="14">
@@ -30095,7 +30095,7 @@
         <v>0.35</v>
       </c>
       <c r="J14" s="33" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="15">
@@ -30127,7 +30127,7 @@
         <v>0.35</v>
       </c>
       <c r="J15" s="33" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="16">
@@ -30159,7 +30159,7 @@
         <v>0.35</v>
       </c>
       <c r="J16" s="33" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="17">
@@ -30191,7 +30191,7 @@
         <v>0.35</v>
       </c>
       <c r="J17" s="33" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="18">
@@ -30223,7 +30223,7 @@
         <v>0.35</v>
       </c>
       <c r="J18" s="33" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="19">
@@ -30255,7 +30255,7 @@
         <v>0.35</v>
       </c>
       <c r="J19" s="33" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="20">
@@ -30287,7 +30287,7 @@
         <v>0.35</v>
       </c>
       <c r="J20" s="33" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="21">
@@ -30319,7 +30319,7 @@
         <v>0.35</v>
       </c>
       <c r="J21" s="33" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="22">
@@ -30351,7 +30351,7 @@
         <v>0.35</v>
       </c>
       <c r="J22" s="33" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="23">
@@ -30383,7 +30383,7 @@
         <v>0.35</v>
       </c>
       <c r="J23" s="33" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="24">
@@ -30415,7 +30415,7 @@
         <v>0.35</v>
       </c>
       <c r="J24" s="33" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="25">
@@ -30444,10 +30444,10 @@
         <v>0.326</v>
       </c>
       <c r="I25" s="33" t="n">
-        <v>0.377</v>
+        <v>0.375</v>
       </c>
       <c r="J25" s="33" t="n">
-        <v>1</v>
+        <v>0.905</v>
       </c>
     </row>
     <row r="26">
@@ -30476,10 +30476,10 @@
         <v>0.351</v>
       </c>
       <c r="I26" s="33" t="n">
-        <v>0.403</v>
+        <v>0.4</v>
       </c>
       <c r="J26" s="33" t="n">
-        <v>1</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="27">
@@ -30508,10 +30508,10 @@
         <v>0.377</v>
       </c>
       <c r="I27" s="33" t="n">
-        <v>0.43</v>
+        <v>0.425</v>
       </c>
       <c r="J27" s="33" t="n">
-        <v>1</v>
+        <v>0.915</v>
       </c>
     </row>
     <row r="28">
@@ -30540,10 +30540,10 @@
         <v>0.403</v>
       </c>
       <c r="I28" s="33" t="n">
-        <v>0.457</v>
+        <v>0.45</v>
       </c>
       <c r="J28" s="33" t="n">
-        <v>1</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="29">
@@ -30572,10 +30572,10 @@
         <v>0.429</v>
       </c>
       <c r="I29" s="33" t="n">
-        <v>0.483</v>
+        <v>0.475</v>
       </c>
       <c r="J29" s="33" t="n">
-        <v>1</v>
+        <v>0.925</v>
       </c>
     </row>
     <row r="30">
@@ -30604,10 +30604,10 @@
         <v>0.454</v>
       </c>
       <c r="I30" s="33" t="n">
-        <v>0.51</v>
+        <v>0.5</v>
       </c>
       <c r="J30" s="33" t="n">
-        <v>1</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="31">
@@ -30636,10 +30636,10 @@
         <v>0.48</v>
       </c>
       <c r="I31" s="33" t="n">
-        <v>0.537</v>
+        <v>0.525</v>
       </c>
       <c r="J31" s="33" t="n">
-        <v>1</v>
+        <v>0.9350000000000001</v>
       </c>
     </row>
     <row r="32">
@@ -30668,10 +30668,10 @@
         <v>0.506</v>
       </c>
       <c r="I32" s="33" t="n">
-        <v>0.5629999999999999</v>
+        <v>0.55</v>
       </c>
       <c r="J32" s="33" t="n">
-        <v>1</v>
+        <v>0.9399999999999999</v>
       </c>
     </row>
     <row r="33">
@@ -30700,10 +30700,10 @@
         <v>0.531</v>
       </c>
       <c r="I33" s="33" t="n">
-        <v>0.59</v>
+        <v>0.575</v>
       </c>
       <c r="J33" s="33" t="n">
-        <v>1</v>
+        <v>0.945</v>
       </c>
     </row>
     <row r="34">
@@ -30732,10 +30732,10 @@
         <v>0.5570000000000001</v>
       </c>
       <c r="I34" s="33" t="n">
-        <v>0.617</v>
+        <v>0.6</v>
       </c>
       <c r="J34" s="33" t="n">
-        <v>1</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="35">
@@ -30764,10 +30764,10 @@
         <v>0.583</v>
       </c>
       <c r="I35" s="33" t="n">
-        <v>0.643</v>
+        <v>0.625</v>
       </c>
       <c r="J35" s="33" t="n">
-        <v>1</v>
+        <v>0.955</v>
       </c>
     </row>
     <row r="36">
@@ -30796,10 +30796,10 @@
         <v>0.609</v>
       </c>
       <c r="I36" s="33" t="n">
-        <v>0.67</v>
+        <v>0.65</v>
       </c>
       <c r="J36" s="33" t="n">
-        <v>1</v>
+        <v>0.96</v>
       </c>
     </row>
     <row r="37">
@@ -30828,10 +30828,10 @@
         <v>0.634</v>
       </c>
       <c r="I37" s="33" t="n">
-        <v>0.697</v>
+        <v>0.675</v>
       </c>
       <c r="J37" s="33" t="n">
-        <v>1</v>
+        <v>0.965</v>
       </c>
     </row>
     <row r="38">
@@ -30860,10 +30860,10 @@
         <v>0.66</v>
       </c>
       <c r="I38" s="33" t="n">
-        <v>0.723</v>
+        <v>0.7</v>
       </c>
       <c r="J38" s="33" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="39">
@@ -30892,10 +30892,10 @@
         <v>0.6860000000000001</v>
       </c>
       <c r="I39" s="33" t="n">
-        <v>0.75</v>
+        <v>0.725</v>
       </c>
       <c r="J39" s="33" t="n">
-        <v>1</v>
+        <v>0.975</v>
       </c>
     </row>
     <row r="40">
@@ -30924,10 +30924,10 @@
         <v>0.711</v>
       </c>
       <c r="I40" s="33" t="n">
-        <v>0.777</v>
+        <v>0.75</v>
       </c>
       <c r="J40" s="33" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="41">
@@ -30956,10 +30956,10 @@
         <v>0.737</v>
       </c>
       <c r="I41" s="33" t="n">
-        <v>0.803</v>
+        <v>0.775</v>
       </c>
       <c r="J41" s="33" t="n">
-        <v>1</v>
+        <v>0.985</v>
       </c>
     </row>
     <row r="42">
@@ -30988,10 +30988,10 @@
         <v>0.763</v>
       </c>
       <c r="I42" s="33" t="n">
-        <v>0.83</v>
+        <v>0.8</v>
       </c>
       <c r="J42" s="33" t="n">
-        <v>1</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="43">
@@ -31020,10 +31020,10 @@
         <v>0.789</v>
       </c>
       <c r="I43" s="33" t="n">
-        <v>0.857</v>
+        <v>0.825</v>
       </c>
       <c r="J43" s="33" t="n">
-        <v>1</v>
+        <v>0.995</v>
       </c>
     </row>
     <row r="44">
@@ -31052,7 +31052,7 @@
         <v>0.8139999999999999</v>
       </c>
       <c r="I44" s="33" t="n">
-        <v>0.883</v>
+        <v>0.85</v>
       </c>
       <c r="J44" s="33" t="n">
         <v>1</v>
@@ -31084,7 +31084,7 @@
         <v>0.84</v>
       </c>
       <c r="I45" s="33" t="n">
-        <v>0.91</v>
+        <v>0.875</v>
       </c>
       <c r="J45" s="33" t="n">
         <v>1</v>
@@ -31116,7 +31116,7 @@
         <v>0.866</v>
       </c>
       <c r="I46" s="33" t="n">
-        <v>0.9370000000000001</v>
+        <v>0.9</v>
       </c>
       <c r="J46" s="33" t="n">
         <v>1</v>
@@ -31148,7 +31148,7 @@
         <v>0.891</v>
       </c>
       <c r="I47" s="33" t="n">
-        <v>0.963</v>
+        <v>0.925</v>
       </c>
       <c r="J47" s="33" t="n">
         <v>1</v>
@@ -31180,7 +31180,7 @@
         <v>0.917</v>
       </c>
       <c r="I48" s="33" t="n">
-        <v>0.99</v>
+        <v>0.95</v>
       </c>
       <c r="J48" s="33" t="n">
         <v>1</v>
@@ -31212,7 +31212,7 @@
         <v>0.9429999999999999</v>
       </c>
       <c r="I49" s="33" t="n">
-        <v>1.017</v>
+        <v>0.975</v>
       </c>
       <c r="J49" s="33" t="n">
         <v>1</v>
@@ -31244,7 +31244,7 @@
         <v>0.969</v>
       </c>
       <c r="I50" s="33" t="n">
-        <v>1.043</v>
+        <v>1</v>
       </c>
       <c r="J50" s="33" t="n">
         <v>1</v>
@@ -31276,7 +31276,7 @@
         <v>0.994</v>
       </c>
       <c r="I51" s="33" t="n">
-        <v>1.07</v>
+        <v>1.025</v>
       </c>
       <c r="J51" s="33" t="n">
         <v>1</v>
@@ -31308,7 +31308,7 @@
         <v>1.02</v>
       </c>
       <c r="I52" s="33" t="n">
-        <v>1.097</v>
+        <v>1.05</v>
       </c>
       <c r="J52" s="33" t="n">
         <v>1</v>
@@ -31340,7 +31340,7 @@
         <v>1.046</v>
       </c>
       <c r="I53" s="33" t="n">
-        <v>1.123</v>
+        <v>1.075</v>
       </c>
       <c r="J53" s="33" t="n">
         <v>1</v>
@@ -31372,7 +31372,7 @@
         <v>1.071</v>
       </c>
       <c r="I54" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J54" s="33" t="n">
         <v>1</v>
@@ -31404,7 +31404,7 @@
         <v>1.097</v>
       </c>
       <c r="I55" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J55" s="33" t="n">
         <v>1</v>
@@ -31436,7 +31436,7 @@
         <v>1.123</v>
       </c>
       <c r="I56" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J56" s="33" t="n">
         <v>1</v>
@@ -31468,7 +31468,7 @@
         <v>1.149</v>
       </c>
       <c r="I57" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J57" s="33" t="n">
         <v>1</v>
@@ -31500,7 +31500,7 @@
         <v>1.174</v>
       </c>
       <c r="I58" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J58" s="33" t="n">
         <v>1</v>
@@ -31532,7 +31532,7 @@
         <v>1.2</v>
       </c>
       <c r="I59" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J59" s="33" t="n">
         <v>1</v>
@@ -31564,7 +31564,7 @@
         <v>1.2</v>
       </c>
       <c r="I60" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J60" s="33" t="n">
         <v>1</v>
@@ -31596,7 +31596,7 @@
         <v>1.2</v>
       </c>
       <c r="I61" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J61" s="33" t="n">
         <v>1</v>
@@ -31628,7 +31628,7 @@
         <v>1.2</v>
       </c>
       <c r="I62" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J62" s="33" t="n">
         <v>1</v>
@@ -31660,7 +31660,7 @@
         <v>1.2</v>
       </c>
       <c r="I63" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J63" s="33" t="n">
         <v>1</v>
@@ -31692,7 +31692,7 @@
         <v>1.2</v>
       </c>
       <c r="I64" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J64" s="33" t="n">
         <v>1</v>
@@ -31724,7 +31724,7 @@
         <v>1.2</v>
       </c>
       <c r="I65" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J65" s="33" t="n">
         <v>1</v>
@@ -31756,7 +31756,7 @@
         <v>1.2</v>
       </c>
       <c r="I66" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J66" s="33" t="n">
         <v>1</v>
@@ -31788,7 +31788,7 @@
         <v>1.2</v>
       </c>
       <c r="I67" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J67" s="33" t="n">
         <v>1</v>
@@ -31820,7 +31820,7 @@
         <v>1.2</v>
       </c>
       <c r="I68" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J68" s="33" t="n">
         <v>1</v>
@@ -31852,7 +31852,7 @@
         <v>1.2</v>
       </c>
       <c r="I69" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J69" s="33" t="n">
         <v>1</v>
@@ -31884,7 +31884,7 @@
         <v>1.2</v>
       </c>
       <c r="I70" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J70" s="33" t="n">
         <v>1</v>
@@ -31916,7 +31916,7 @@
         <v>1.2</v>
       </c>
       <c r="I71" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J71" s="33" t="n">
         <v>1</v>
@@ -31948,7 +31948,7 @@
         <v>1.2</v>
       </c>
       <c r="I72" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J72" s="33" t="n">
         <v>1</v>
@@ -31980,7 +31980,7 @@
         <v>1.2</v>
       </c>
       <c r="I73" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J73" s="33" t="n">
         <v>1</v>
@@ -32012,7 +32012,7 @@
         <v>1.2</v>
       </c>
       <c r="I74" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J74" s="33" t="n">
         <v>1</v>
@@ -32044,7 +32044,7 @@
         <v>1.2</v>
       </c>
       <c r="I75" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J75" s="33" t="n">
         <v>1</v>
@@ -32076,7 +32076,7 @@
         <v>1.2</v>
       </c>
       <c r="I76" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J76" s="33" t="n">
         <v>1</v>
@@ -32108,7 +32108,7 @@
         <v>1.2</v>
       </c>
       <c r="I77" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J77" s="33" t="n">
         <v>1</v>
@@ -32140,7 +32140,7 @@
         <v>1.2</v>
       </c>
       <c r="I78" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J78" s="33" t="n">
         <v>1</v>
@@ -32172,7 +32172,7 @@
         <v>1.2</v>
       </c>
       <c r="I79" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J79" s="33" t="n">
         <v>1</v>
@@ -32204,7 +32204,7 @@
         <v>1.2</v>
       </c>
       <c r="I80" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J80" s="33" t="n">
         <v>1</v>
@@ -32236,7 +32236,7 @@
         <v>1.2</v>
       </c>
       <c r="I81" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J81" s="33" t="n">
         <v>1</v>
@@ -32268,7 +32268,7 @@
         <v>1.2</v>
       </c>
       <c r="I82" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J82" s="33" t="n">
         <v>1</v>
@@ -32300,7 +32300,7 @@
         <v>1.2</v>
       </c>
       <c r="I83" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J83" s="33" t="n">
         <v>1</v>
@@ -32332,7 +32332,7 @@
         <v>1.2</v>
       </c>
       <c r="I84" s="33" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="J84" s="33" t="n">
         <v>1</v>
@@ -32364,7 +32364,7 @@
         <v>1.2</v>
       </c>
       <c r="I85" s="33" t="n">
-        <v>1.142</v>
+        <v>1.093</v>
       </c>
       <c r="J85" s="33" t="n">
         <v>1</v>
@@ -32396,7 +32396,7 @@
         <v>1.2</v>
       </c>
       <c r="I86" s="33" t="n">
-        <v>1.133</v>
+        <v>1.087</v>
       </c>
       <c r="J86" s="33" t="n">
         <v>1</v>
@@ -32428,7 +32428,7 @@
         <v>1.2</v>
       </c>
       <c r="I87" s="33" t="n">
-        <v>1.125</v>
+        <v>1.08</v>
       </c>
       <c r="J87" s="33" t="n">
         <v>1</v>
@@ -32460,7 +32460,7 @@
         <v>1.2</v>
       </c>
       <c r="I88" s="33" t="n">
-        <v>1.117</v>
+        <v>1.073</v>
       </c>
       <c r="J88" s="33" t="n">
         <v>1</v>
@@ -32492,7 +32492,7 @@
         <v>1.2</v>
       </c>
       <c r="I89" s="33" t="n">
-        <v>1.108</v>
+        <v>1.067</v>
       </c>
       <c r="J89" s="33" t="n">
         <v>1</v>
@@ -32524,7 +32524,7 @@
         <v>1.2</v>
       </c>
       <c r="I90" s="33" t="n">
-        <v>1.1</v>
+        <v>1.06</v>
       </c>
       <c r="J90" s="33" t="n">
         <v>1</v>
@@ -32556,7 +32556,7 @@
         <v>1.2</v>
       </c>
       <c r="I91" s="33" t="n">
-        <v>1.092</v>
+        <v>1.053</v>
       </c>
       <c r="J91" s="33" t="n">
         <v>1</v>
@@ -32588,7 +32588,7 @@
         <v>1.2</v>
       </c>
       <c r="I92" s="33" t="n">
-        <v>1.083</v>
+        <v>1.047</v>
       </c>
       <c r="J92" s="33" t="n">
         <v>1</v>
@@ -32620,7 +32620,7 @@
         <v>1.2</v>
       </c>
       <c r="I93" s="33" t="n">
-        <v>1.075</v>
+        <v>1.04</v>
       </c>
       <c r="J93" s="33" t="n">
         <v>1</v>
@@ -32652,7 +32652,7 @@
         <v>1.2</v>
       </c>
       <c r="I94" s="33" t="n">
-        <v>1.067</v>
+        <v>1.033</v>
       </c>
       <c r="J94" s="33" t="n">
         <v>1</v>
@@ -32684,7 +32684,7 @@
         <v>1.2</v>
       </c>
       <c r="I95" s="33" t="n">
-        <v>1.058</v>
+        <v>1.027</v>
       </c>
       <c r="J95" s="33" t="n">
         <v>1</v>
@@ -32716,7 +32716,7 @@
         <v>1.2</v>
       </c>
       <c r="I96" s="33" t="n">
-        <v>1.05</v>
+        <v>1.02</v>
       </c>
       <c r="J96" s="33" t="n">
         <v>1</v>
@@ -32748,7 +32748,7 @@
         <v>1.2</v>
       </c>
       <c r="I97" s="33" t="n">
-        <v>1.042</v>
+        <v>1.013</v>
       </c>
       <c r="J97" s="33" t="n">
         <v>1</v>
@@ -32780,7 +32780,7 @@
         <v>1.2</v>
       </c>
       <c r="I98" s="33" t="n">
-        <v>1.033</v>
+        <v>1.007</v>
       </c>
       <c r="J98" s="33" t="n">
         <v>1</v>
@@ -32812,7 +32812,7 @@
         <v>1.2</v>
       </c>
       <c r="I99" s="33" t="n">
-        <v>1.025</v>
+        <v>1</v>
       </c>
       <c r="J99" s="33" t="n">
         <v>1</v>
@@ -32844,7 +32844,7 @@
         <v>1.18</v>
       </c>
       <c r="I100" s="33" t="n">
-        <v>1.017</v>
+        <v>0.993</v>
       </c>
       <c r="J100" s="33" t="n">
         <v>1</v>
@@ -32876,7 +32876,7 @@
         <v>1.16</v>
       </c>
       <c r="I101" s="33" t="n">
-        <v>1.008</v>
+        <v>0.987</v>
       </c>
       <c r="J101" s="33" t="n">
         <v>1</v>
@@ -32908,7 +32908,7 @@
         <v>1.14</v>
       </c>
       <c r="I102" s="33" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="J102" s="33" t="n">
         <v>1</v>
@@ -32940,7 +32940,7 @@
         <v>1.12</v>
       </c>
       <c r="I103" s="33" t="n">
-        <v>0.992</v>
+        <v>0.973</v>
       </c>
       <c r="J103" s="33" t="n">
         <v>1</v>
@@ -32972,7 +32972,7 @@
         <v>1.1</v>
       </c>
       <c r="I104" s="33" t="n">
-        <v>0.983</v>
+        <v>0.967</v>
       </c>
       <c r="J104" s="33" t="n">
         <v>1</v>
@@ -33004,7 +33004,7 @@
         <v>1.08</v>
       </c>
       <c r="I105" s="33" t="n">
-        <v>0.975</v>
+        <v>0.96</v>
       </c>
       <c r="J105" s="33" t="n">
         <v>1</v>
@@ -33036,7 +33036,7 @@
         <v>1.06</v>
       </c>
       <c r="I106" s="33" t="n">
-        <v>0.967</v>
+        <v>0.953</v>
       </c>
       <c r="J106" s="33" t="n">
         <v>1</v>
@@ -33068,7 +33068,7 @@
         <v>1.04</v>
       </c>
       <c r="I107" s="33" t="n">
-        <v>0.958</v>
+        <v>0.947</v>
       </c>
       <c r="J107" s="33" t="n">
         <v>1</v>
@@ -33100,7 +33100,7 @@
         <v>1.02</v>
       </c>
       <c r="I108" s="33" t="n">
-        <v>0.95</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="J108" s="33" t="n">
         <v>1</v>
@@ -33132,7 +33132,7 @@
         <v>1</v>
       </c>
       <c r="I109" s="33" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="J109" s="33" t="n">
         <v>1</v>
@@ -33164,7 +33164,7 @@
         <v>0.98</v>
       </c>
       <c r="I110" s="33" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.927</v>
       </c>
       <c r="J110" s="33" t="n">
         <v>1</v>
@@ -33196,7 +33196,7 @@
         <v>0.96</v>
       </c>
       <c r="I111" s="33" t="n">
-        <v>0.925</v>
+        <v>0.92</v>
       </c>
       <c r="J111" s="33" t="n">
         <v>1</v>
@@ -33228,7 +33228,7 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="I112" s="33" t="n">
-        <v>0.917</v>
+        <v>0.913</v>
       </c>
       <c r="J112" s="33" t="n">
         <v>1</v>
@@ -33260,7 +33260,7 @@
         <v>0.92</v>
       </c>
       <c r="I113" s="33" t="n">
-        <v>0.908</v>
+        <v>0.907</v>
       </c>
       <c r="J113" s="33" t="n">
         <v>1</v>

</xml_diff>